<commit_message>
Added ASHD with 148 households dataset
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -58,11 +58,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -429,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,10 +502,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="3" t="n">
         <v>40444</v>
       </c>
       <c r="G2" t="inlineStr">
@@ -543,10 +545,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="3" t="n">
         <v>41455</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -559,7 +561,6 @@
           <t>30 minute</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -582,10 +583,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,10 +626,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G5" t="inlineStr">
@@ -668,10 +669,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="3" t="n">
         <v>41455</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -684,7 +685,6 @@
           <t>30 minute</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -707,10 +707,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G7" t="inlineStr">
@@ -750,10 +750,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -793,10 +793,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G9" t="inlineStr">
@@ -836,10 +836,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G10" t="inlineStr">
@@ -879,10 +879,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G11" t="inlineStr">
@@ -922,10 +922,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G12" t="inlineStr">
@@ -965,10 +965,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G13" t="inlineStr">
@@ -1008,10 +1008,10 @@
           <t>Ausgrid, BOM weather data</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="3" t="n">
         <v>41455</v>
       </c>
       <c r="G14" t="inlineStr">
@@ -1051,10 +1051,10 @@
           <t>Ausgrid, BOM weather data, solcast data</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F15" s="3" t="n">
         <v>41455</v>
       </c>
       <c r="G15" t="inlineStr">
@@ -1094,10 +1094,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="3" t="n">
         <v>38473</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="3" t="n">
         <v>45412</v>
       </c>
       <c r="G16" t="inlineStr">
@@ -1137,10 +1137,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="3" t="n">
         <v>44013</v>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="F17" s="3" t="n">
         <v>45107</v>
       </c>
       <c r="G17" t="inlineStr">
@@ -1297,6 +1297,135 @@
       <c r="I20" t="inlineStr">
         <is>
           <t>Generated for publication/journal_article_1 from 100 selected BESS households; 30-minute values are arithmetic mean power, not summed energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ds19_ashd_148hh</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Ausgrid Solar Home Dataset, aggregate of the 148 households nearest to Sydney Airport based on postcode centroid distance</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>netload_kW</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Ausgrid</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>40360</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>41455.97916666666</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Selected from the 300 ASHD households using postcode centroid distance to Sydney Airport BOM station 066037; selected-household audit is stored beside the processing notebook in ignored_from_git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ds20_ashd_148hh_with_weather</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ds19 enhanced with BOM Sydney Airport weather data</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Ausgrid, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>40360</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>41455.97916666666</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Uses Sydney Airport BOM station 066037 and the same weather variables as AEDP ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ds21_ashd_148hh_with_weather_cloud_solcast</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ds20 enhanced with Solcast Sydney Airport cloud opacity data</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h, cloud_opacity</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ausgrid, BOM weather data, solcast data</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>40360</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>41455.97916666666</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>cloud_opacity is a continuous Solcast value from 0 to 100, where 0 means no cloud and 100 means completely cloudy.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
major folder restructure for paper 1, and started preparing notebooks to run paper data creation and experiments
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -58,13 +58,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -431,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,10 +500,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="2" t="n">
         <v>40360</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="2" t="n">
         <v>40444</v>
       </c>
       <c r="G2" t="inlineStr">
@@ -545,10 +543,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="2" t="n">
         <v>40360</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="2" t="n">
         <v>41455</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -561,6 +559,7 @@
           <t>30 minute</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -583,10 +582,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="2" t="n">
         <v>44378</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -626,10 +625,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="2" t="n">
         <v>44378</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G5" t="inlineStr">
@@ -669,10 +668,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="2" t="n">
         <v>40360</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F6" s="2" t="n">
         <v>41455</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -685,6 +684,7 @@
           <t>30 minute</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -707,10 +707,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="2" t="n">
         <v>44378</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G7" t="inlineStr">
@@ -750,10 +750,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="2" t="n">
         <v>44378</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -793,10 +793,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="2" t="n">
         <v>44378</v>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="F9" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G9" t="inlineStr">
@@ -836,10 +836,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="2" t="n">
         <v>44378</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G10" t="inlineStr">
@@ -879,10 +879,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="2" t="n">
         <v>44378</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G11" t="inlineStr">
@@ -922,10 +922,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="2" t="n">
         <v>44378</v>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="F12" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G12" t="inlineStr">
@@ -965,10 +965,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="2" t="n">
         <v>44378</v>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="F13" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G13" t="inlineStr">
@@ -1008,10 +1008,10 @@
           <t>Ausgrid, BOM weather data</t>
         </is>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="2" t="n">
         <v>40360</v>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="2" t="n">
         <v>41455</v>
       </c>
       <c r="G14" t="inlineStr">
@@ -1051,10 +1051,10 @@
           <t>Ausgrid, BOM weather data, solcast data</t>
         </is>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="2" t="n">
         <v>40360</v>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="F15" s="2" t="n">
         <v>41455</v>
       </c>
       <c r="G15" t="inlineStr">
@@ -1094,10 +1094,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="2" t="n">
         <v>38473</v>
       </c>
-      <c r="F16" s="3" t="n">
+      <c r="F16" s="2" t="n">
         <v>45412</v>
       </c>
       <c r="G16" t="inlineStr">
@@ -1137,10 +1137,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="E17" s="2" t="n">
         <v>44013</v>
       </c>
-      <c r="F17" s="3" t="n">
+      <c r="F17" s="2" t="n">
         <v>45107</v>
       </c>
       <c r="G17" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Generated for publication/journal_article_1 from 100 selected BESS households; 30-minute values are arithmetic mean power, not summed energy.</t>
+          <t>Generated for publication/journal_article_1 from 100 selected BESS households; 30-minute values are arithmetic mean power, not summed energy. Exploratory 100-household SA BESS aggregate. Retained for diagnostics; 56 of the 100 selected households contain meaningful negative reconstructed underlying-load intervals below -0.05 kW.</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Generated for publication/journal_article_1 from 100 selected BESS households; 30-minute values are arithmetic mean power, not summed energy.</t>
+          <t>Generated for publication/journal_article_1 from 100 selected BESS households; 30-minute values are arithmetic mean power, not summed energy. Exploratory 100-household SA BESS aggregate. Retained for diagnostics; 56 of the 100 selected households contain meaningful negative reconstructed underlying-load intervals below -0.05 kW.</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Generated for publication/journal_article_1 from 100 selected BESS households; 30-minute values are arithmetic mean power, not summed energy.</t>
+          <t>Generated for publication/journal_article_1 from 100 selected BESS households; 30-minute values are arithmetic mean power, not summed energy. Exploratory 100-household SA BESS aggregate. Retained for diagnostics; 56 of the 100 selected households contain meaningful negative reconstructed underlying-load intervals below -0.05 kW.</t>
         </is>
       </c>
     </row>
@@ -1321,10 +1321,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="2" t="n">
         <v>40360</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="F21" s="2" t="n">
         <v>41455.97916666666</v>
       </c>
       <c r="G21" t="inlineStr">
@@ -1364,10 +1364,10 @@
           <t>Ausgrid, BOM weather data</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="E22" s="2" t="n">
         <v>40360</v>
       </c>
-      <c r="F22" s="4" t="n">
+      <c r="F22" s="2" t="n">
         <v>41455.97916666666</v>
       </c>
       <c r="G22" t="inlineStr">
@@ -1407,10 +1407,10 @@
           <t>Ausgrid, BOM weather data, solcast data</t>
         </is>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="2" t="n">
         <v>40360</v>
       </c>
-      <c r="F23" s="4" t="n">
+      <c r="F23" s="2" t="n">
         <v>41455.97916666666</v>
       </c>
       <c r="G23" t="inlineStr">
@@ -1426,6 +1426,2027 @@
       <c r="I23" t="inlineStr">
         <is>
           <t>cloud_opacity is a continuous Solcast value from 0 to 100, where 0 means no cloud and 100 means completely cloudy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ds22_sa_bess_44hh_pos_underlying_load_30min</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Solar Analytics CICCADA BESS aggregate of 44 households with no meaningful negative underlying-load intervals, underlying load, 30-minute mean power.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>netload_kW</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Solar Analytics CICCADA BESS</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2024-02-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2025-02-24 23:30:00</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Selected from the 100-household SA BESS cohort using meaningful_negative_underlying_load_count_post_fill == 0 at the -0.05 kW threshold; 30-minute values are arithmetic mean power, not summed energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ds23_sa_bess_44hh_pos_net_load_with_pv_30min</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Solar Analytics CICCADA BESS aggregate of 44 households with no meaningful negative underlying-load intervals, net load with PV, 30-minute mean power.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>netload_kW</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Solar Analytics CICCADA BESS</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2024-02-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2025-02-24 23:30:00</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Selected from the 100-household SA BESS cohort using meaningful_negative_underlying_load_count_post_fill == 0 at the -0.05 kW threshold; 30-minute values are arithmetic mean power, not summed energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ds24_sa_bess_44hh_pos_net_load_with_pv_battery_30min</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Solar Analytics CICCADA BESS aggregate of 44 households with no meaningful negative underlying-load intervals, net load with PV and battery, 30-minute mean power.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>netload_kW</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Solar Analytics CICCADA BESS</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2024-02-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2025-02-24 23:30:00</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Selected from the 100-household SA BESS cohort using meaningful_negative_underlying_load_count_post_fill == 0 at the -0.05 kW threshold; 30-minute values are arithmetic mean power, not summed energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ds25_aedp_1hh_sample01_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1 household sample 01, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ds26_aedp_1hh_sample02_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1 household sample 02, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ds27_aedp_1hh_sample03_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1 household sample 03, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ds28_aedp_1hh_sample04_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1 household sample 04, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ds29_aedp_1hh_sample05_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1 household sample 05, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ds30_aedp_1hh_sample06_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1 household sample 06, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ds31_aedp_1hh_sample07_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1 household sample 07, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ds32_aedp_1hh_sample08_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1 household sample 08, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ds33_aedp_1hh_sample09_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1 household sample 09, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ds34_aedp_1hh_sample10_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1 household sample 10, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ds35_aedp_10hh_sample01_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 01, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ds36_aedp_10hh_sample02_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 02, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ds37_aedp_10hh_sample03_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 03, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ds38_aedp_10hh_sample04_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 04, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ds39_aedp_10hh_sample05_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 05, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ds40_aedp_10hh_sample06_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 06, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ds41_aedp_10hh_sample07_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 07, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ds42_aedp_10hh_sample08_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 08, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ds43_aedp_10hh_sample09_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 09, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ds44_aedp_10hh_sample10_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 10, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ds45_aedp_100hh_sample01_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 01, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ds46_aedp_100hh_sample02_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 02, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ds47_aedp_100hh_sample03_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 03, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ds48_aedp_100hh_sample04_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 04, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ds49_aedp_100hh_sample05_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 05, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ds50_aedp_100hh_sample06_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 06, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ds51_aedp_100hh_sample07_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 07, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ds52_aedp_100hh_sample08_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 08, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ds53_aedp_100hh_sample09_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 09, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ds54_aedp_100hh_sample10_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 10, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ds55_aedp_1000hh_sample01_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1000 household sample 01, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ds56_aedp_1000hh_sample02_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1000 household sample 02, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ds57_aedp_1000hh_sample03_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1000 household sample 03, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ds58_aedp_1000hh_sample04_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1000 household sample 04, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ds59_aedp_1000hh_sample05_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1000 household sample 05, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ds60_aedp_1000hh_sample06_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1000 household sample 06, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ds61_aedp_1000hh_sample07_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1000 household sample 07, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ds62_aedp_1000hh_sample08_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1000 household sample 08, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ds63_aedp_1000hh_sample09_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1000 household sample 09, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ds64_aedp_1000hh_sample10_30min_with_weather</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>AEDP aggregation-level publication dataset, 1000 household sample 10, 30-minute net load with Sydney Airport weather.</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>AEDP, BOM weather data</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2021-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2024-06-30 23:30:00</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>30 minute</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
created aedp different aggregation data. WIP running experiment
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$I$38</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,8 +19,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -58,11 +60,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -429,51 +432,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>column</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>start date</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>end date</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>length</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>interval</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -500,10 +503,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="3" t="n">
         <v>40444</v>
       </c>
       <c r="G2" t="inlineStr">
@@ -543,10 +546,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="3" t="n">
         <v>41455</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -559,7 +562,9 @@
           <t>30 minute</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="n">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -582,10 +587,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,10 +630,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G5" t="inlineStr">
@@ -668,10 +673,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="3" t="n">
         <v>41455</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -684,7 +689,9 @@
           <t>30 minute</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -707,10 +714,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G7" t="inlineStr">
@@ -750,10 +757,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -793,10 +800,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G9" t="inlineStr">
@@ -836,10 +843,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G10" t="inlineStr">
@@ -879,10 +886,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G11" t="inlineStr">
@@ -922,10 +929,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G12" t="inlineStr">
@@ -965,10 +972,10 @@
           <t>Solar Analytics, Wattwatchers collected in Darth</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="3" t="n">
         <v>44378</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" s="3" t="n">
         <v>45473</v>
       </c>
       <c r="G13" t="inlineStr">
@@ -1008,10 +1015,10 @@
           <t>Ausgrid, BOM weather data</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="3" t="n">
         <v>41455</v>
       </c>
       <c r="G14" t="inlineStr">
@@ -1051,10 +1058,10 @@
           <t>Ausgrid, BOM weather data, solcast data</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F15" s="3" t="n">
         <v>41455</v>
       </c>
       <c r="G15" t="inlineStr">
@@ -1094,10 +1101,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="3" t="n">
         <v>38473</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="3" t="n">
         <v>45412</v>
       </c>
       <c r="G16" t="inlineStr">
@@ -1137,10 +1144,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="3" t="n">
         <v>44013</v>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="F17" s="3" t="n">
         <v>45107</v>
       </c>
       <c r="G17" t="inlineStr">
@@ -1321,10 +1328,10 @@
           <t>Ausgrid</t>
         </is>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="E21" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="F21" s="3" t="n">
         <v>41455.97916666666</v>
       </c>
       <c r="G21" t="inlineStr">
@@ -1364,10 +1371,10 @@
           <t>Ausgrid, BOM weather data</t>
         </is>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="F22" s="3" t="n">
         <v>41455.97916666666</v>
       </c>
       <c r="G22" t="inlineStr">
@@ -1407,10 +1414,10 @@
           <t>Ausgrid, BOM weather data, solcast data</t>
         </is>
       </c>
-      <c r="E23" s="2" t="n">
+      <c r="E23" s="3" t="n">
         <v>40360</v>
       </c>
-      <c r="F23" s="2" t="n">
+      <c r="F23" s="3" t="n">
         <v>41455.97916666666</v>
       </c>
       <c r="G23" t="inlineStr">
@@ -1591,15 +1598,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E27" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1613,7 +1616,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
@@ -1638,15 +1641,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E28" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1660,7 +1659,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
@@ -1685,15 +1684,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E29" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1707,19 +1702,19 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ds28_aedp_1hh_sample04_30min_with_weather</t>
+          <t>ds28_aedp_10hh_sample01_30min_with_weather</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 1 household sample 04, 30-minute net load with Sydney Airport weather.</t>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 01, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1732,15 +1727,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E30" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1754,19 +1745,19 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ds29_aedp_1hh_sample05_30min_with_weather</t>
+          <t>ds29_aedp_10hh_sample02_30min_with_weather</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 1 household sample 05, 30-minute net load with Sydney Airport weather.</t>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 02, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1779,15 +1770,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E31" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1801,19 +1788,19 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ds30_aedp_1hh_sample06_30min_with_weather</t>
+          <t>ds30_aedp_10hh_sample03_30min_with_weather</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 1 household sample 06, 30-minute net load with Sydney Airport weather.</t>
+          <t>AEDP aggregation-level publication dataset, 10 household sample 03, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1826,15 +1813,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E32" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1848,19 +1831,19 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ds31_aedp_1hh_sample07_30min_with_weather</t>
+          <t>ds31_aedp_100hh_sample01_30min_with_weather</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 1 household sample 07, 30-minute net load with Sydney Airport weather.</t>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 01, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1873,15 +1856,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E33" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1895,19 +1874,19 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ds32_aedp_1hh_sample08_30min_with_weather</t>
+          <t>ds32_aedp_100hh_sample02_30min_with_weather</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 1 household sample 08, 30-minute net load with Sydney Airport weather.</t>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 02, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1920,15 +1899,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E34" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1942,19 +1917,19 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ds33_aedp_1hh_sample09_30min_with_weather</t>
+          <t>ds33_aedp_100hh_sample03_30min_with_weather</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 1 household sample 09, 30-minute net load with Sydney Airport weather.</t>
+          <t>AEDP aggregation-level publication dataset, 100 household sample 03, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1967,15 +1942,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E35" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1989,19 +1960,19 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled without replacement within the group from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ds34_aedp_1hh_sample10_30min_with_weather</t>
+          <t>ds34_aedp_1000hh_sample01_30min_with_weather</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 1 household sample 10, 30-minute net load with Sydney Airport weather.</t>
+          <t>AEDP aggregation-level publication dataset, synthetic-bootstrap 1000 household sample 01, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2014,15 +1985,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E36" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2036,19 +2003,19 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled with replacement from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ds35_aedp_10hh_sample01_30min_with_weather</t>
+          <t>ds35_aedp_1000hh_sample02_30min_with_weather</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 01, 30-minute net load with Sydney Airport weather.</t>
+          <t>AEDP aggregation-level publication dataset, synthetic-bootstrap 1000 household sample 02, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2061,15 +2028,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E37" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2083,19 +2046,19 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled with replacement from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ds36_aedp_10hh_sample02_30min_with_weather</t>
+          <t>ds36_aedp_1000hh_sample03_30min_with_weather</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 02, 30-minute net load with Sydney Airport weather.</t>
+          <t>AEDP aggregation-level publication dataset, synthetic-bootstrap 1000 household sample 03, 30-minute net load with Sydney Airport weather.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2108,15 +2071,11 @@
           <t>AEDP, BOM weather data</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
+      <c r="E38" s="3" t="n">
+        <v>44378</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>45473.97916666666</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2130,1327 +2089,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>ds37_aedp_10hh_sample03_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 03, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>ds38_aedp_10hh_sample04_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 04, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>ds39_aedp_10hh_sample05_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 05, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>ds40_aedp_10hh_sample06_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 06, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>ds41_aedp_10hh_sample07_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 07, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>ds42_aedp_10hh_sample08_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 08, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>ds43_aedp_10hh_sample09_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 09, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>ds44_aedp_10hh_sample10_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 10 household sample 10, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>ds45_aedp_100hh_sample01_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 01, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>ds46_aedp_100hh_sample02_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 02, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>ds47_aedp_100hh_sample03_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 03, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>ds48_aedp_100hh_sample04_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 04, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>ds49_aedp_100hh_sample05_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 05, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>ds50_aedp_100hh_sample06_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 06, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>ds51_aedp_100hh_sample07_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 07, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>ds52_aedp_100hh_sample08_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 08, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>ds53_aedp_100hh_sample09_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 09, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>ds54_aedp_100hh_sample10_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 100 household sample 10, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>ds55_aedp_1000hh_sample01_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 1000 household sample 01, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>ds56_aedp_1000hh_sample02_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 1000 household sample 02, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>ds57_aedp_1000hh_sample03_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 1000 household sample 03, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>ds58_aedp_1000hh_sample04_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 1000 household sample 04, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>ds59_aedp_1000hh_sample05_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 1000 household sample 05, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>ds60_aedp_1000hh_sample06_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 1000 household sample 06, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>ds61_aedp_1000hh_sample07_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 1000 household sample 07, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>ds62_aedp_1000hh_sample08_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 1000 household sample 08, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>ds63_aedp_1000hh_sample09_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 1000 household sample 09, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>ds64_aedp_1000hh_sample10_30min_with_weather</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>AEDP aggregation-level publication dataset, 1000 household sample 10, 30-minute net load with Sydney Airport weather.</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>netload_kW, air_temperature_in_degrees_c, relative_humidity_in_percentage, wind_speed_in_km_h</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>AEDP, BOM weather data</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>2021-07-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>2024-06-30 23:30:00</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>30 minute</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level with fixed random seed 20260521; includes Sydney Airport weather variables matching ds11. The 1000-household sample is synthetic and bootstrapped with replacement from the 148-household AEDP cohort.</t>
+          <t>Generated by publication/journal_article_1/notebooks/03_aedp_aggregation_level/2.1_build_aedp_site_30min_checkpoints.ipynb and 2.2_generate_aedp_aggregation_datasets.ipynb with fixed random seed 20260521; sampled with replacement from the 139 valid AEDP per-household checkpoints; household series are forward-filled before aggregation; includes Sydney Airport weather variables matching ds11.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>